<commit_message>
Redesign warehouse inventory: category allowlist, id extract, surplus report
Replace product_inventory schema with 3-column موجودی انبار (category_code,
item_code_desc, quantity). Extract id from item text, filter by DB
category_codes allowlist, default priority 1 and drop priority 0.
Restructure upload menu (inventory submenu + add 4-digit code), rename
labels to موجودی روزانه سایت / مصرف ماهیانه, and add گزارش مواد مازاد.
</commit_message>
<xml_diff>
--- a/samples/02_product_inventory.xlsx
+++ b/samples/02_product_inventory.xlsx
@@ -413,298 +413,100 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>domain</t>
+          <t>کد دسته بندی</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>tundish_type</t>
+          <t>کد و شرح کالا</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>assignee_id</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>assignee_name</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>product_name</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>quantity</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>location</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>notes</t>
+          <t>موجودی</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>خط-A</t>
+          <t>1201</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>تاندیش اسلب</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1001</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>علی رضایی</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>اسید سولفوریک</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
+          <t>ACID01 - اسید سولفوریک</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>20</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>لیتر</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>قفسه ۱</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>کم</t>
-        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>خط-A</t>
+          <t>1201</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>تاندیش بلوم</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1001</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>علی رضایی</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>سود سوزآور</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
+          <t>CAUST02 - سود سوزآور</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>80</v>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>کیلو</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>قفسه ۲</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>خط-B</t>
+          <t>1201</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>تاندیش بلوم</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1002</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>مریم احمدی</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>آب اکسیژنه</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
+          <t>H2O203 - آب اکسیژنه</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>100</v>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>لیتر</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>سالن B</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>خط-B</t>
+          <t>1201</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>تاندیش اسلب</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1003</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>حسین کریمی</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>کلر</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
+          <t>CL04 - کلر</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>8</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>کیلو</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>سالن B</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>بحرانی</t>
-        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>انبار</t>
+          <t>1201</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>تاندیش بیلت</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1002</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>مریم احمدی</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>روغن صنعتی</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>50</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>لیتر</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>انبار مرکزی</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
+          <t>OIL05 - روغن صنعتی</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>500</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>